<commit_message>
Pour publication (#55) 752d9a4541855a1c3fe4257075faa8f454d7ea8e
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-tddui-bundle.xlsx
+++ b/ig/main/StructureDefinition-tddui-bundle.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0-ballot</t>
+    <t>1.0.1-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-12T16:43:27+00:00</t>
+    <t>2024-02-13T13:14:14+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>